<commit_message>
AUT-683 Make client name and short name mandatory, test fix
</commit_message>
<xml_diff>
--- a/tara-admin-import/src/test/resources/import_files/client-with-min-fields.xlsx
+++ b/tara-admin-import/src/test/resources/import_files/client-with-min-fields.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mari-Nicole.Berezovs\c\dev-aut\TARA-GovSSO-Admin\tara-admin-import\src\test\resources\import_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mari-Nicole.Berezovs\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5497402-364F-4A61-B90C-B8CB0934E286}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E722C3BE-C907-4DAB-A0C4-A9B1578B7185}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="30600" yWindow="-120" windowWidth="30960" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>Institution name</t>
   </si>
@@ -103,6 +103,9 @@
   </si>
   <si>
     <t>sn_et</t>
+  </si>
+  <si>
+    <t>n_et</t>
   </si>
 </sst>
 </file>
@@ -657,7 +660,9 @@
       <c r="E2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="G2" s="1"/>
+      <c r="G2" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="J2" s="3" t="s">
         <v>25</v>
       </c>

</xml_diff>